<commit_message>
Still trying to learn to use Git
</commit_message>
<xml_diff>
--- a/gallup_confidence_military/Gallup_Confidence_Military_1991-2016.xlsx
+++ b/gallup_confidence_military/Gallup_Confidence_Military_1991-2016.xlsx
@@ -1,26 +1,39 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10531"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10621"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/james-macbook/Data/dissertation/gallup_confidence_military/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E70B5FC5-A1B8-C347-8AAD-F1A555F779A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{585CC4F7-9A2B-1944-A8C6-2ABE966C1EC6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4420" yWindow="660" windowWidth="25820" windowHeight="17940" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Military" sheetId="4" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="36">
   <si>
     <t>Time</t>
   </si>
@@ -125,6 +138,9 @@
   </si>
   <si>
     <t>1990</t>
+  </si>
+  <si>
+    <t>Agg</t>
   </si>
 </sst>
 </file>
@@ -478,13 +494,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I36"/>
+  <dimension ref="A1:J36"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="9" width="20"/>
+    <col min="1" max="3" width="20"/>
+    <col min="5" max="10" width="20"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -495,25 +512,28 @@
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="E1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -524,25 +544,29 @@
         <v>0.32</v>
       </c>
       <c r="D2" s="2">
+        <f>SUM(B2:C2)</f>
+        <v>0.73</v>
+      </c>
+      <c r="E2" s="2">
         <v>0.19</v>
       </c>
-      <c r="E2" s="2">
+      <c r="F2" s="2">
         <v>7.0000000000000007E-2</v>
       </c>
-      <c r="F2" s="2">
-        <v>0</v>
-      </c>
       <c r="G2" s="2">
-        <v>0.01</v>
+        <v>0</v>
       </c>
       <c r="H2" s="2">
-        <v>0</v>
-      </c>
-      <c r="I2" s="3">
+        <v>0.01</v>
+      </c>
+      <c r="I2" s="2">
+        <v>0</v>
+      </c>
+      <c r="J2" s="3">
         <v>1027</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>10</v>
       </c>
@@ -553,25 +577,29 @@
         <v>0.3</v>
       </c>
       <c r="D3" s="2">
+        <f t="shared" ref="D3:D27" si="0">SUM(B3:C3)</f>
+        <v>0.72</v>
+      </c>
+      <c r="E3" s="2">
         <v>0.19</v>
       </c>
-      <c r="E3" s="2">
+      <c r="F3" s="2">
         <v>0.06</v>
       </c>
-      <c r="F3" s="2">
-        <v>0.01</v>
-      </c>
       <c r="G3" s="2">
         <v>0.01</v>
       </c>
       <c r="H3" s="2">
-        <v>0</v>
-      </c>
-      <c r="I3" s="3">
+        <v>0.01</v>
+      </c>
+      <c r="I3" s="2">
+        <v>0</v>
+      </c>
+      <c r="J3" s="3">
         <v>1527</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>11</v>
       </c>
@@ -582,25 +610,29 @@
         <v>0.35</v>
       </c>
       <c r="D4" s="2">
+        <f t="shared" si="0"/>
+        <v>0.74</v>
+      </c>
+      <c r="E4" s="2">
         <v>0.2</v>
       </c>
-      <c r="E4" s="2">
+      <c r="F4" s="2">
         <v>0.06</v>
       </c>
-      <c r="F4" s="2">
-        <v>0.01</v>
-      </c>
       <c r="G4" s="2">
-        <v>0</v>
+        <v>0.01</v>
       </c>
       <c r="H4" s="2">
         <v>0</v>
       </c>
-      <c r="I4" s="3">
+      <c r="I4" s="2">
+        <v>0</v>
+      </c>
+      <c r="J4" s="3">
         <v>1027</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>12</v>
       </c>
@@ -611,25 +643,29 @@
         <v>0.33</v>
       </c>
       <c r="D5" s="2">
+        <f t="shared" si="0"/>
+        <v>0.76</v>
+      </c>
+      <c r="E5" s="2">
         <v>0.17</v>
       </c>
-      <c r="E5" s="2">
+      <c r="F5" s="2">
         <v>0.06</v>
       </c>
-      <c r="F5" s="2">
-        <v>0</v>
-      </c>
       <c r="G5" s="2">
         <v>0</v>
       </c>
       <c r="H5" s="2">
         <v>0</v>
       </c>
-      <c r="I5" s="3">
+      <c r="I5" s="2">
+        <v>0</v>
+      </c>
+      <c r="J5" s="3">
         <v>1529</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>13</v>
       </c>
@@ -640,25 +676,29 @@
         <v>0.32</v>
       </c>
       <c r="D6" s="2">
+        <f t="shared" si="0"/>
+        <v>0.75</v>
+      </c>
+      <c r="E6" s="2">
         <v>0.18</v>
       </c>
-      <c r="E6" s="2">
+      <c r="F6" s="2">
         <v>0.05</v>
       </c>
-      <c r="F6" s="2">
-        <v>0.01</v>
-      </c>
       <c r="G6" s="2">
         <v>0.01</v>
       </c>
       <c r="H6" s="2">
-        <v>0</v>
-      </c>
-      <c r="I6" s="3">
+        <v>0.01</v>
+      </c>
+      <c r="I6" s="2">
+        <v>0</v>
+      </c>
+      <c r="J6" s="3">
         <v>1004</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>14</v>
       </c>
@@ -669,25 +709,29 @@
         <v>0.31</v>
       </c>
       <c r="D7" s="2">
+        <f t="shared" si="0"/>
+        <v>0.78</v>
+      </c>
+      <c r="E7" s="2">
         <v>0.16</v>
       </c>
-      <c r="E7" s="2">
+      <c r="F7" s="2">
         <v>0.03</v>
       </c>
-      <c r="F7" s="2">
-        <v>0</v>
-      </c>
       <c r="G7" s="2">
-        <v>0.01</v>
+        <v>0</v>
       </c>
       <c r="H7" s="2">
-        <v>0</v>
-      </c>
-      <c r="I7" s="3">
+        <v>0.01</v>
+      </c>
+      <c r="I7" s="2">
+        <v>0</v>
+      </c>
+      <c r="J7" s="3">
         <v>1020</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>15</v>
       </c>
@@ -698,25 +742,29 @@
         <v>0.32</v>
       </c>
       <c r="D8" s="2">
+        <f t="shared" si="0"/>
+        <v>0.76</v>
+      </c>
+      <c r="E8" s="2">
         <v>0.18</v>
       </c>
-      <c r="E8" s="2">
+      <c r="F8" s="2">
         <v>0.04</v>
       </c>
-      <c r="F8" s="2">
-        <v>0.01</v>
-      </c>
       <c r="G8" s="2">
         <v>0.01</v>
       </c>
       <c r="H8" s="2">
         <v>0.01</v>
       </c>
-      <c r="I8" s="3">
+      <c r="I8" s="2">
+        <v>0.01</v>
+      </c>
+      <c r="J8" s="3">
         <v>1020</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>16</v>
       </c>
@@ -727,25 +775,29 @@
         <v>0.37</v>
       </c>
       <c r="D9" s="2">
+        <f t="shared" si="0"/>
+        <v>0.82000000000000006</v>
+      </c>
+      <c r="E9" s="2">
         <v>0.12</v>
       </c>
-      <c r="E9" s="2">
+      <c r="F9" s="2">
         <v>0.05</v>
       </c>
-      <c r="F9" s="2">
-        <v>0</v>
-      </c>
       <c r="G9" s="2">
-        <v>0.01</v>
+        <v>0</v>
       </c>
       <c r="H9" s="2">
-        <v>0</v>
-      </c>
-      <c r="I9" s="3">
+        <v>0.01</v>
+      </c>
+      <c r="I9" s="2">
+        <v>0</v>
+      </c>
+      <c r="J9" s="3">
         <v>1011</v>
       </c>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>17</v>
       </c>
@@ -756,25 +808,29 @@
         <v>0.26</v>
       </c>
       <c r="D10" s="2">
+        <f t="shared" si="0"/>
+        <v>0.71</v>
+      </c>
+      <c r="E10" s="2">
         <v>0.2</v>
       </c>
-      <c r="E10" s="2">
+      <c r="F10" s="2">
         <v>7.0000000000000007E-2</v>
       </c>
-      <c r="F10" s="2">
-        <v>0.01</v>
-      </c>
       <c r="G10" s="2">
         <v>0.01</v>
       </c>
       <c r="H10" s="2">
         <v>0.01</v>
       </c>
-      <c r="I10" s="3">
+      <c r="I10" s="2">
+        <v>0.01</v>
+      </c>
+      <c r="J10" s="3">
         <v>822</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>18</v>
       </c>
@@ -785,25 +841,29 @@
         <v>0.3</v>
       </c>
       <c r="D11" s="2">
+        <f t="shared" si="0"/>
+        <v>0.69</v>
+      </c>
+      <c r="E11" s="2">
         <v>0.21</v>
       </c>
-      <c r="E11" s="2">
+      <c r="F11" s="2">
         <v>0.08</v>
       </c>
-      <c r="F11" s="2">
-        <v>0.01</v>
-      </c>
       <c r="G11" s="2">
-        <v>0</v>
+        <v>0.01</v>
       </c>
       <c r="H11" s="2">
         <v>0</v>
       </c>
-      <c r="I11" s="3">
+      <c r="I11" s="2">
+        <v>0</v>
+      </c>
+      <c r="J11" s="3">
         <v>1007</v>
       </c>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>19</v>
       </c>
@@ -814,25 +874,29 @@
         <v>0.32</v>
       </c>
       <c r="D12" s="2">
+        <f t="shared" si="0"/>
+        <v>0.73</v>
+      </c>
+      <c r="E12" s="2">
         <v>0.19</v>
       </c>
-      <c r="E12" s="2">
+      <c r="F12" s="2">
         <v>0.05</v>
       </c>
-      <c r="F12" s="2">
-        <v>0.01</v>
-      </c>
       <c r="G12" s="2">
         <v>0.01</v>
       </c>
       <c r="H12" s="2">
-        <v>0</v>
-      </c>
-      <c r="I12" s="3">
+        <v>0.01</v>
+      </c>
+      <c r="I12" s="2">
+        <v>0</v>
+      </c>
+      <c r="J12" s="3">
         <v>1002</v>
       </c>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>20</v>
       </c>
@@ -843,25 +907,29 @@
         <v>0.32</v>
       </c>
       <c r="D13" s="2">
+        <f t="shared" si="0"/>
+        <v>0.74</v>
+      </c>
+      <c r="E13" s="2">
         <v>0.18</v>
       </c>
-      <c r="E13" s="2">
+      <c r="F13" s="2">
         <v>7.0000000000000007E-2</v>
       </c>
-      <c r="F13" s="2">
-        <v>0.01</v>
-      </c>
       <c r="G13" s="2">
-        <v>0</v>
+        <v>0.01</v>
       </c>
       <c r="H13" s="2">
         <v>0</v>
       </c>
-      <c r="I13" s="3">
+      <c r="I13" s="2">
+        <v>0</v>
+      </c>
+      <c r="J13" s="3">
         <v>1004</v>
       </c>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>21</v>
       </c>
@@ -872,25 +940,29 @@
         <v>0.39</v>
       </c>
       <c r="D14" s="2">
+        <f t="shared" si="0"/>
+        <v>0.75</v>
+      </c>
+      <c r="E14" s="2">
         <v>0.19</v>
       </c>
-      <c r="E14" s="2">
+      <c r="F14" s="2">
         <v>0.05</v>
       </c>
-      <c r="F14" s="2">
-        <v>0</v>
-      </c>
       <c r="G14" s="2">
         <v>0</v>
       </c>
       <c r="H14" s="2">
         <v>0</v>
       </c>
-      <c r="I14" s="3">
+      <c r="I14" s="2">
+        <v>0</v>
+      </c>
+      <c r="J14" s="3">
         <v>1002</v>
       </c>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>22</v>
       </c>
@@ -901,23 +973,27 @@
         <v>0.34</v>
       </c>
       <c r="D15" s="2">
+        <f t="shared" si="0"/>
+        <v>0.82000000000000006</v>
+      </c>
+      <c r="E15" s="2">
         <v>0.14000000000000001</v>
       </c>
-      <c r="E15" s="2">
+      <c r="F15" s="2">
         <v>0.04</v>
       </c>
-      <c r="F15" s="2">
-        <v>0</v>
-      </c>
       <c r="G15" s="2">
         <v>0</v>
       </c>
-      <c r="H15" s="2"/>
-      <c r="I15" s="3">
+      <c r="H15" s="2">
+        <v>0</v>
+      </c>
+      <c r="I15" s="2"/>
+      <c r="J15" s="3">
         <v>1029</v>
       </c>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>23</v>
       </c>
@@ -928,25 +1004,29 @@
         <v>0.36</v>
       </c>
       <c r="D16" s="2">
+        <f t="shared" si="0"/>
+        <v>0.78</v>
+      </c>
+      <c r="E16" s="2">
         <v>0.16</v>
       </c>
-      <c r="E16" s="2">
+      <c r="F16" s="2">
         <v>0.04</v>
       </c>
-      <c r="F16" s="2">
-        <v>0</v>
-      </c>
       <c r="G16" s="2">
         <v>0</v>
       </c>
       <c r="H16" s="2">
         <v>0</v>
       </c>
-      <c r="I16" s="3">
+      <c r="I16" s="2">
+        <v>0</v>
+      </c>
+      <c r="J16" s="3">
         <v>1020</v>
       </c>
     </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>24</v>
       </c>
@@ -957,23 +1037,27 @@
         <v>0.34</v>
       </c>
       <c r="D17" s="2">
+        <f t="shared" si="0"/>
+        <v>0.66</v>
+      </c>
+      <c r="E17" s="2">
         <v>0.24</v>
       </c>
-      <c r="E17" s="2">
+      <c r="F17" s="2">
         <v>0.06</v>
       </c>
-      <c r="F17" s="2">
+      <c r="G17" s="2">
         <v>0.03</v>
       </c>
-      <c r="G17" s="2">
+      <c r="H17" s="2">
         <v>0.02</v>
       </c>
-      <c r="H17" s="2"/>
-      <c r="I17" s="3">
+      <c r="I17" s="2"/>
+      <c r="J17" s="3">
         <v>1011</v>
       </c>
     </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>25</v>
       </c>
@@ -984,23 +1068,27 @@
         <v>0.39</v>
       </c>
       <c r="D18" s="2">
+        <f t="shared" si="0"/>
+        <v>0.63</v>
+      </c>
+      <c r="E18" s="2">
         <v>0.26</v>
       </c>
-      <c r="E18" s="2">
+      <c r="F18" s="2">
         <v>7.0000000000000007E-2</v>
       </c>
-      <c r="F18" s="2">
-        <v>0.01</v>
-      </c>
       <c r="G18" s="2">
+        <v>0.01</v>
+      </c>
+      <c r="H18" s="2">
         <v>0.02</v>
       </c>
-      <c r="H18" s="2"/>
-      <c r="I18" s="3">
+      <c r="I18" s="2"/>
+      <c r="J18" s="3">
         <v>1021</v>
       </c>
     </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>26</v>
       </c>
@@ -1011,23 +1099,27 @@
         <v>0.34</v>
       </c>
       <c r="D19" s="2">
+        <f t="shared" si="0"/>
+        <v>0.68</v>
+      </c>
+      <c r="E19" s="2">
         <v>0.25</v>
       </c>
-      <c r="E19" s="2">
+      <c r="F19" s="2">
         <v>0.06</v>
       </c>
-      <c r="F19" s="2">
-        <v>0</v>
-      </c>
       <c r="G19" s="2">
         <v>0</v>
       </c>
-      <c r="H19" s="2"/>
-      <c r="I19" s="3">
+      <c r="H19" s="2">
+        <v>0</v>
+      </c>
+      <c r="I19" s="2"/>
+      <c r="J19" s="3">
         <v>1016</v>
       </c>
     </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>27</v>
       </c>
@@ -1038,23 +1130,27 @@
         <v>0.31</v>
       </c>
       <c r="D20" s="2">
+        <f t="shared" si="0"/>
+        <v>0.64</v>
+      </c>
+      <c r="E20" s="2">
         <v>0.25</v>
       </c>
-      <c r="E20" s="2">
+      <c r="F20" s="2">
         <v>0.09</v>
       </c>
-      <c r="F20" s="2">
-        <v>0.01</v>
-      </c>
       <c r="G20" s="2">
+        <v>0.01</v>
+      </c>
+      <c r="H20" s="2">
         <v>0.02</v>
       </c>
-      <c r="H20" s="2"/>
-      <c r="I20" s="3">
+      <c r="I20" s="2"/>
+      <c r="J20" s="3">
         <v>1003</v>
       </c>
     </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>28</v>
       </c>
@@ -1065,23 +1161,27 @@
         <v>0.3</v>
       </c>
       <c r="D21" s="2">
+        <f t="shared" si="0"/>
+        <v>0.6</v>
+      </c>
+      <c r="E21" s="2">
         <v>0.27</v>
       </c>
-      <c r="E21" s="2">
+      <c r="F21" s="2">
         <v>0.1</v>
-      </c>
-      <c r="F21" s="2">
-        <v>0.02</v>
       </c>
       <c r="G21" s="2">
         <v>0.02</v>
       </c>
-      <c r="H21" s="2"/>
-      <c r="I21" s="3">
+      <c r="H21" s="2">
+        <v>0.02</v>
+      </c>
+      <c r="I21" s="2"/>
+      <c r="J21" s="3">
         <v>1004</v>
       </c>
     </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>29</v>
       </c>
@@ -1092,23 +1192,27 @@
         <v>0.36</v>
       </c>
       <c r="D22" s="2">
+        <f t="shared" si="0"/>
+        <v>0.65999999999999992</v>
+      </c>
+      <c r="E22" s="2">
         <v>0.25</v>
       </c>
-      <c r="E22" s="2">
+      <c r="F22" s="2">
         <v>7.0000000000000007E-2</v>
       </c>
-      <c r="F22" s="2">
-        <v>0</v>
-      </c>
       <c r="G22" s="2">
+        <v>0</v>
+      </c>
+      <c r="H22" s="2">
         <v>0.02</v>
       </c>
-      <c r="H22" s="2"/>
-      <c r="I22" s="3">
+      <c r="I22" s="2"/>
+      <c r="J22" s="3">
         <v>1019</v>
       </c>
     </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
         <v>30</v>
       </c>
@@ -1119,23 +1223,27 @@
         <v>0.31</v>
       </c>
       <c r="D23" s="2">
+        <f t="shared" si="0"/>
+        <v>0.64</v>
+      </c>
+      <c r="E23" s="2">
         <v>0.27</v>
       </c>
-      <c r="E23" s="2">
+      <c r="F23" s="2">
         <v>7.0000000000000007E-2</v>
       </c>
-      <c r="F23" s="2">
-        <v>0.01</v>
-      </c>
       <c r="G23" s="2">
         <v>0.01</v>
       </c>
-      <c r="H23" s="2"/>
-      <c r="I23" s="3">
+      <c r="H23" s="2">
+        <v>0.01</v>
+      </c>
+      <c r="I23" s="2"/>
+      <c r="J23" s="3">
         <v>1008</v>
       </c>
     </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
         <v>31</v>
       </c>
@@ -1146,23 +1254,27 @@
         <v>0.33</v>
       </c>
       <c r="D24" s="2">
+        <f t="shared" si="0"/>
+        <v>0.63</v>
+      </c>
+      <c r="E24" s="2">
         <v>0.26</v>
       </c>
-      <c r="E24" s="2">
+      <c r="F24" s="2">
         <v>0.08</v>
       </c>
-      <c r="F24" s="2">
-        <v>0.01</v>
-      </c>
       <c r="G24" s="2">
+        <v>0.01</v>
+      </c>
+      <c r="H24" s="2">
         <v>0.02</v>
       </c>
-      <c r="H24" s="2"/>
-      <c r="I24" s="3">
+      <c r="I24" s="2"/>
+      <c r="J24" s="3">
         <v>1036</v>
       </c>
     </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
         <v>32</v>
       </c>
@@ -1173,23 +1285,27 @@
         <v>0.35</v>
       </c>
       <c r="D25" s="2">
+        <f t="shared" si="0"/>
+        <v>0.66999999999999993</v>
+      </c>
+      <c r="E25" s="2">
         <v>0.22</v>
       </c>
-      <c r="E25" s="2">
+      <c r="F25" s="2">
         <v>0.08</v>
       </c>
-      <c r="F25" s="2">
-        <v>0.01</v>
-      </c>
       <c r="G25" s="2">
         <v>0.01</v>
       </c>
-      <c r="H25" s="2"/>
-      <c r="I25" s="3">
+      <c r="H25" s="2">
+        <v>0.01</v>
+      </c>
+      <c r="I25" s="2"/>
+      <c r="J25" s="3">
         <v>1003</v>
       </c>
     </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
         <v>33</v>
       </c>
@@ -1200,23 +1316,27 @@
         <v>0.34</v>
       </c>
       <c r="D26" s="2">
+        <f t="shared" si="0"/>
+        <v>0.78</v>
+      </c>
+      <c r="E26" s="2">
         <v>0.15</v>
       </c>
-      <c r="E26" s="2">
+      <c r="F26" s="2">
         <v>0.05</v>
       </c>
-      <c r="F26" s="2">
-        <v>0</v>
-      </c>
       <c r="G26" s="2">
+        <v>0</v>
+      </c>
+      <c r="H26" s="2">
         <v>0.02</v>
       </c>
-      <c r="H26" s="2"/>
-      <c r="I26" s="3">
+      <c r="I26" s="2"/>
+      <c r="J26" s="3">
         <v>2012</v>
       </c>
     </row>
-    <row r="27" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
         <v>34</v>
       </c>
@@ -1227,23 +1347,27 @@
         <v>0.31</v>
       </c>
       <c r="D27" s="2">
+        <f t="shared" si="0"/>
+        <v>0.67999999999999994</v>
+      </c>
+      <c r="E27" s="2">
         <v>0.22</v>
       </c>
-      <c r="E27" s="2">
+      <c r="F27" s="2">
         <v>7.0000000000000007E-2</v>
       </c>
-      <c r="F27" s="2">
-        <v>0.01</v>
-      </c>
       <c r="G27" s="2">
+        <v>0.01</v>
+      </c>
+      <c r="H27" s="2">
         <v>0.02</v>
       </c>
-      <c r="H27" s="2"/>
-      <c r="I27" s="3">
+      <c r="I27" s="2"/>
+      <c r="J27" s="3">
         <v>1241</v>
       </c>
     </row>
-    <row r="28" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:10" x14ac:dyDescent="0.2">
       <c r="B28" s="2"/>
       <c r="C28" s="2"/>
       <c r="D28" s="2"/>
@@ -1251,9 +1375,10 @@
       <c r="F28" s="2"/>
       <c r="G28" s="2"/>
       <c r="H28" s="2"/>
-      <c r="I28" s="3"/>
-    </row>
-    <row r="29" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="I28" s="2"/>
+      <c r="J28" s="3"/>
+    </row>
+    <row r="29" spans="1:10" x14ac:dyDescent="0.2">
       <c r="B29" s="2"/>
       <c r="C29" s="2"/>
       <c r="D29" s="2"/>
@@ -1261,9 +1386,10 @@
       <c r="F29" s="2"/>
       <c r="G29" s="2"/>
       <c r="H29" s="2"/>
-      <c r="I29" s="3"/>
-    </row>
-    <row r="30" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="I29" s="2"/>
+      <c r="J29" s="3"/>
+    </row>
+    <row r="30" spans="1:10" x14ac:dyDescent="0.2">
       <c r="B30" s="2"/>
       <c r="C30" s="2"/>
       <c r="D30" s="2"/>
@@ -1271,9 +1397,10 @@
       <c r="F30" s="2"/>
       <c r="G30" s="2"/>
       <c r="H30" s="2"/>
-      <c r="I30" s="3"/>
-    </row>
-    <row r="31" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="I30" s="2"/>
+      <c r="J30" s="3"/>
+    </row>
+    <row r="31" spans="1:10" x14ac:dyDescent="0.2">
       <c r="B31" s="2"/>
       <c r="C31" s="2"/>
       <c r="D31" s="2"/>
@@ -1281,9 +1408,10 @@
       <c r="F31" s="2"/>
       <c r="G31" s="2"/>
       <c r="H31" s="2"/>
-      <c r="I31" s="3"/>
-    </row>
-    <row r="32" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="I31" s="2"/>
+      <c r="J31" s="3"/>
+    </row>
+    <row r="32" spans="1:10" x14ac:dyDescent="0.2">
       <c r="B32" s="2"/>
       <c r="C32" s="2"/>
       <c r="D32" s="2"/>
@@ -1291,9 +1419,10 @@
       <c r="F32" s="2"/>
       <c r="G32" s="2"/>
       <c r="H32" s="2"/>
-      <c r="I32" s="3"/>
-    </row>
-    <row r="33" spans="2:9" x14ac:dyDescent="0.2">
+      <c r="I32" s="2"/>
+      <c r="J32" s="3"/>
+    </row>
+    <row r="33" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B33" s="2"/>
       <c r="C33" s="2"/>
       <c r="D33" s="2"/>
@@ -1301,9 +1430,10 @@
       <c r="F33" s="2"/>
       <c r="G33" s="2"/>
       <c r="H33" s="2"/>
-      <c r="I33" s="3"/>
-    </row>
-    <row r="34" spans="2:9" x14ac:dyDescent="0.2">
+      <c r="I33" s="2"/>
+      <c r="J33" s="3"/>
+    </row>
+    <row r="34" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B34" s="2"/>
       <c r="C34" s="2"/>
       <c r="D34" s="2"/>
@@ -1311,9 +1441,10 @@
       <c r="F34" s="2"/>
       <c r="G34" s="2"/>
       <c r="H34" s="2"/>
-      <c r="I34" s="3"/>
-    </row>
-    <row r="35" spans="2:9" x14ac:dyDescent="0.2">
+      <c r="I34" s="2"/>
+      <c r="J34" s="3"/>
+    </row>
+    <row r="35" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B35" s="2"/>
       <c r="C35" s="2"/>
       <c r="D35" s="2"/>
@@ -1321,9 +1452,10 @@
       <c r="F35" s="2"/>
       <c r="G35" s="2"/>
       <c r="H35" s="2"/>
-      <c r="I35" s="3"/>
-    </row>
-    <row r="36" spans="2:9" x14ac:dyDescent="0.2">
+      <c r="I35" s="2"/>
+      <c r="J35" s="3"/>
+    </row>
+    <row r="36" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B36" s="2"/>
       <c r="C36" s="2"/>
       <c r="D36" s="2"/>
@@ -1331,7 +1463,8 @@
       <c r="F36" s="2"/>
       <c r="G36" s="2"/>
       <c r="H36" s="2"/>
-      <c r="I36" s="3"/>
+      <c r="I36" s="2"/>
+      <c r="J36" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>